<commit_message>
Final: add pictures etc
</commit_message>
<xml_diff>
--- a/Expense_Claim_MASTER.xlsx
+++ b/Expense_Claim_MASTER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrien Partier\Downloads\HKUST\Vsceptre Expense Claim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF5077D-44E5-4267-B544-F5B206084B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE60000D-B273-4C7C-BC55-D30991D08879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>Item</t>
   </si>
@@ -250,6 +250,9 @@
   <si>
     <t>Category / Categories</t>
   </si>
+  <si>
+    <t>Receipt Uploads</t>
+  </si>
 </sst>
 </file>
 
@@ -331,7 +334,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -628,12 +631,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -660,6 +672,84 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -672,7 +762,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -687,107 +777,35 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1057,7 +1075,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA975"/>
+  <dimension ref="A1:AA976"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.08984375" style="4" customWidth="1"/>
@@ -1080,11 +1098,11 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="H1" s="11"/>
-      <c r="I1" s="12"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="38"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -1105,9 +1123,9 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G2" s="13"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="41"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -1134,9 +1152,9 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="41"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -1163,9 +1181,9 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="18"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="44"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -1193,8 +1211,8 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -1215,26 +1233,26 @@
       <c r="AA5" s="1"/>
     </row>
     <row r="6" spans="1:27" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="28"/>
-      <c r="G6" s="26" t="s">
+      <c r="F6" s="47"/>
+      <c r="G6" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="27" t="s">
+      <c r="H6" s="28" t="s">
         <v>5</v>
       </c>
       <c r="I6" s="29"/>
@@ -1258,17 +1276,17 @@
       <c r="AA6" s="1"/>
     </row>
     <row r="7" spans="1:27" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="30">
+      <c r="A7" s="15">
         <v>1</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="47"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="48"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="27"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -1289,18 +1307,18 @@
       <c r="AA7" s="2"/>
     </row>
     <row r="8" spans="1:27" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="27" t="s">
+      <c r="B8" s="46"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
       <c r="I8" s="29"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
@@ -1322,21 +1340,21 @@
       <c r="AA8" s="2"/>
     </row>
     <row r="9" spans="1:27" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="33" t="str" cm="1">
+      <c r="A9" s="50" t="str" cm="1">
         <f t="array" ref="A9">IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($G$7:$G$7,($G$7:$G$7&lt;&gt;"")*($H$7:$H$7&lt;&gt;0))),ROWS($A$9:A9)),"")</f>
         <v/>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36" t="str">
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="51"/>
+      <c r="E9" s="30" t="str">
         <f>IF(A9="","",IF(SUMIF($G$7:$G$7,A9,$H$7:$H$7)=0,"",SUMIF($G$7:$G$7,A9,$H$7:$H$7)))</f>
         <v/>
       </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="37"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="32"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -1357,20 +1375,20 @@
       <c r="AA9" s="2"/>
     </row>
     <row r="10" spans="1:27" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="41">
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="33">
         <f>SUM($H$7:$H$7)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="42"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="35"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -1391,19 +1409,19 @@
       <c r="AA10" s="2"/>
     </row>
     <row r="11" spans="1:27" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44" t="s">
+      <c r="B11" s="22"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
-      <c r="I11" s="44"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1424,19 +1442,19 @@
       <c r="AA11" s="2"/>
     </row>
     <row r="12" spans="1:27" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="45" t="s">
+      <c r="A12" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1457,17 +1475,17 @@
       <c r="AA12" s="2"/>
     </row>
     <row r="13" spans="1:27" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="45" t="s">
+      <c r="A13" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="44"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1546,7 +1564,7 @@
       <c r="AA15" s="2"/>
     </row>
     <row r="16" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="12" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="3"/>
@@ -1577,19 +1595,19 @@
       <c r="AA16" s="2"/>
     </row>
     <row r="17" spans="1:27" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="20">
+      <c r="A17" s="10">
         <v>1</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
@@ -1610,7 +1628,7 @@
       <c r="AA17" s="2"/>
     </row>
     <row r="18" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="21">
+      <c r="A18" s="11">
         <v>2</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -1646,16 +1664,16 @@
       <c r="A19" s="9">
         <v>3</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -1679,16 +1697,16 @@
       <c r="A20" s="9">
         <v>4</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
@@ -1708,16 +1726,16 @@
       <c r="Z20" s="2"/>
       <c r="AA20" s="2"/>
     </row>
-    <row r="21" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
+    <row r="21" spans="1:27" ht="15.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="53"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="53"/>
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+      <c r="I21" s="53"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -1737,16 +1755,16 @@
       <c r="Z21" s="2"/>
       <c r="AA21" s="2"/>
     </row>
-    <row r="22" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
+    <row r="22" spans="1:27" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="54"/>
+      <c r="B22" s="54"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54"/>
+      <c r="G22" s="54"/>
+      <c r="H22" s="54"/>
+      <c r="I22" s="54"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -1795,7 +1813,18 @@
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
     </row>
-    <row r="24" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:27" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="34"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="35"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
@@ -1836,15 +1865,6 @@
       <c r="AA25" s="2"/>
     </row>
     <row r="26" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -2009,7 +2029,7 @@
       <c r="Z31" s="2"/>
       <c r="AA31" s="2"/>
     </row>
-    <row r="32" spans="1:27" ht="9.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -29385,19 +29405,38 @@
       <c r="Z975" s="2"/>
       <c r="AA975" s="2"/>
     </row>
+    <row r="976" spans="1:27" ht="9.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A976" s="3"/>
+      <c r="B976" s="3"/>
+      <c r="C976" s="3"/>
+      <c r="D976" s="3"/>
+      <c r="E976" s="3"/>
+      <c r="F976" s="3"/>
+      <c r="G976" s="3"/>
+      <c r="H976" s="3"/>
+      <c r="I976" s="3"/>
+      <c r="J976" s="2"/>
+      <c r="K976" s="2"/>
+      <c r="L976" s="2"/>
+      <c r="M976" s="2"/>
+      <c r="N976" s="2"/>
+      <c r="O976" s="2"/>
+      <c r="P976" s="2"/>
+      <c r="Q976" s="2"/>
+      <c r="R976" s="2"/>
+      <c r="S976" s="2"/>
+      <c r="T976" s="2"/>
+      <c r="U976" s="2"/>
+      <c r="V976" s="2"/>
+      <c r="W976" s="2"/>
+      <c r="X976" s="2"/>
+      <c r="Y976" s="2"/>
+      <c r="Z976" s="2"/>
+      <c r="AA976" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="E10:I10"/>
+  <mergeCells count="19">
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="G1:I4"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A10:D10"/>
@@ -29405,13 +29444,27 @@
     <mergeCell ref="E8:I8"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="E9:I9"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
   </mergeCells>
-  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125978" footer="0.31496062992125978"/>
-  <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="22" max="16383" man="1"/>
+  </rowBreaks>
   <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1683" yWindow="654" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" xWindow="1683" yWindow="654" count="1">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Category" error="Please select a category from the dropdown list." promptTitle="Expense Category" prompt="Select one of the available expense categories." xr:uid="{99391868-A915-49A4-ACFB-92D1F1BB0C7F}">
           <x14:formula1>
             <xm:f>Dropdown!$A$1:$A$37</xm:f>

</xml_diff>